<commit_message>
Nuevas Minutas de Reunión
</commit_message>
<xml_diff>
--- a/outputs/20261029/DIARCO_Bloque1_Plan_v0.4.xlsx
+++ b/outputs/20261029/DIARCO_Bloque1_Plan_v0.4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PROYECTOS\ETL\CNX_BLOQUE1\outputs\20261029\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23729D4D-AB93-4AB2-9B83-F87BC4F31162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4279963D-F5F5-4B07-A585-35FA09239106}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Resumen" sheetId="1" r:id="rId1"/>
@@ -4143,62 +4143,23 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="21">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="8"/>
-        <color theme="9" tint="-0.249977111117893"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF203040"/>
-        <name val="Arial"/>
-        <scheme val="none"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C260F"/>
@@ -4310,6 +4271,45 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="8"/>
+        <color theme="9" tint="-0.249977111117893"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF203040"/>
+        <name val="Arial"/>
+        <scheme val="none"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -4597,8 +4597,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="T_UAT" displayName="T_UAT" ref="A5:Y38" totalsRowShown="0">
   <tableColumns count="25">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="Caso / ejecución" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Módulo" dataDxfId="1"/>
-    <tableColumn id="25" xr3:uid="{1AA0A8C3-6507-4B4C-B9B1-480310E9F872}" name="Detalle" dataDxfId="0">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="Módulo" dataDxfId="10"/>
+    <tableColumn id="25" xr3:uid="{1AA0A8C3-6507-4B4C-B9B1-480310E9F872}" name="Detalle" dataDxfId="9">
       <calculatedColumnFormula>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0400-000003000000}" name="Escenario"/>
@@ -4650,11 +4650,11 @@
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="17" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="T_Formacion" displayName="T_Formacion" ref="A5:L28" totalsRowShown="0">
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="Módulo" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{41108109-5168-4533-9361-3005560D2281}" name="Descripcion" dataDxfId="9">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="Módulo" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{41108109-5168-4533-9361-3005560D2281}" name="Descripcion" dataDxfId="7">
       <calculatedColumnFormula>VLOOKUP(T_Formacion[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Rol" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="Rol" dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0600-000003000000}" name="Persona"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0600-000004000000}" name="Qué debe demostrar"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0600-000005000000}" name="Versión / material"/>
@@ -4905,7 +4905,7 @@
   <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="43" customWidth="1"/>
+    <col min="1" max="1" width="46.25" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="100" customWidth="1"/>
     <col min="3" max="6" width="12" customWidth="1"/>
   </cols>
@@ -7860,7 +7860,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="O6:O15">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="Falta"/>
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Falta"/>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" sqref="C6:C15" xr:uid="{00000000-0002-0000-0100-000000000000}">
@@ -12781,10 +12781,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J6:J117">
-    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="Bloqueado"/>
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Bloqueado"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P6:P117">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Falta"/>
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Falta"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="J6:J117" xr:uid="{00000000-0002-0000-0200-000000000000}">
@@ -14569,7 +14569,7 @@
       <c r="B6" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="47" t="str">
+      <c r="C6" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Catálogo y maestros</v>
       </c>
@@ -14622,7 +14622,7 @@
       <c r="B7" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="48" t="str">
+      <c r="C7" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Catálogo y maestros</v>
       </c>
@@ -14675,7 +14675,7 @@
       <c r="B8" s="13" t="s">
         <v>48</v>
       </c>
-      <c r="C8" s="47" t="str">
+      <c r="C8" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Surtido, clusters y segmentos</v>
       </c>
@@ -14728,7 +14728,7 @@
       <c r="B9" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="48" t="str">
+      <c r="C9" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Surtido, clusters y segmentos</v>
       </c>
@@ -14781,7 +14781,7 @@
       <c r="B10" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="47" t="str">
+      <c r="C10" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Listas y acuerdos comerciales de compra</v>
       </c>
@@ -14834,7 +14834,7 @@
       <c r="B11" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="C11" s="48" t="str">
+      <c r="C11" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Listas y acuerdos comerciales de compra</v>
       </c>
@@ -14887,7 +14887,7 @@
       <c r="B12" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="C12" s="47" t="str">
+      <c r="C12" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Forecast y compra inteligente/directa</v>
       </c>
@@ -14940,7 +14940,7 @@
       <c r="B13" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="C13" s="48" t="str">
+      <c r="C13" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Forecast y compra inteligente/directa</v>
       </c>
@@ -14993,7 +14993,7 @@
       <c r="B14" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C14" s="47" t="str">
+      <c r="C14" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -15046,7 +15046,7 @@
       <c r="B15" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C15" s="48" t="str">
+      <c r="C15" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -15099,7 +15099,7 @@
       <c r="B16" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C16" s="47" t="str">
+      <c r="C16" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Recepción en sucursal y convivencia SGM</v>
       </c>
@@ -15152,7 +15152,7 @@
       <c r="B17" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C17" s="48" t="str">
+      <c r="C17" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Recepción en sucursal y convivencia SGM</v>
       </c>
@@ -15205,7 +15205,7 @@
       <c r="B18" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="C18" s="47" t="str">
+      <c r="C18" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Inventarios y ajustes</v>
       </c>
@@ -15258,7 +15258,7 @@
       <c r="B19" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="48" t="str">
+      <c r="C19" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Inventarios y ajustes</v>
       </c>
@@ -15311,7 +15311,7 @@
       <c r="B20" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="47" t="str">
+      <c r="C20" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>PDD y necesidades de distribución</v>
       </c>
@@ -15364,7 +15364,7 @@
       <c r="B21" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="C21" s="48" t="str">
+      <c r="C21" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>PDD y necesidades de distribución</v>
       </c>
@@ -15417,7 +15417,7 @@
       <c r="B22" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C22" s="47" t="str">
+      <c r="C22" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Transferencias y distribución con Valkimia</v>
       </c>
@@ -15470,7 +15470,7 @@
       <c r="B23" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="C23" s="48" t="str">
+      <c r="C23" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Transferencias y distribución con Valkimia</v>
       </c>
@@ -15523,7 +15523,7 @@
       <c r="B24" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C24" s="47" t="str">
+      <c r="C24" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Stock, conciliación y observabilidad</v>
       </c>
@@ -15576,7 +15576,7 @@
       <c r="B25" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="48" t="str">
+      <c r="C25" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Stock, conciliación y observabilidad</v>
       </c>
@@ -15629,7 +15629,7 @@
       <c r="B26" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="C26" s="47"/>
+      <c r="C26" s="45"/>
       <c r="D26" s="5" t="s">
         <v>708</v>
       </c>
@@ -15679,7 +15679,7 @@
       <c r="B27" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="C27" s="48"/>
+      <c r="C27" s="46"/>
       <c r="D27" s="6" t="s">
         <v>713</v>
       </c>
@@ -15729,7 +15729,7 @@
       <c r="B28" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="C28" s="47"/>
+      <c r="C28" s="45"/>
       <c r="D28" s="5" t="s">
         <v>718</v>
       </c>
@@ -15779,7 +15779,7 @@
       <c r="B29" s="44" t="s">
         <v>100</v>
       </c>
-      <c r="C29" s="48"/>
+      <c r="C29" s="46"/>
       <c r="D29" s="6" t="s">
         <v>723</v>
       </c>
@@ -15829,7 +15829,7 @@
       <c r="B30" s="43" t="s">
         <v>100</v>
       </c>
-      <c r="C30" s="47"/>
+      <c r="C30" s="45"/>
       <c r="D30" s="5" t="s">
         <v>728</v>
       </c>
@@ -15879,7 +15879,7 @@
       <c r="B31" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C31" s="48" t="str">
+      <c r="C31" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -15932,7 +15932,7 @@
       <c r="B32" s="13" t="s">
         <v>60</v>
       </c>
-      <c r="C32" s="47" t="str">
+      <c r="C32" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -15985,7 +15985,7 @@
       <c r="B33" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C33" s="48" t="str">
+      <c r="C33" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -16038,7 +16038,7 @@
       <c r="B34" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C34" s="47" t="str">
+      <c r="C34" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Transferencias y distribución con Valkimia</v>
       </c>
@@ -16091,7 +16091,7 @@
       <c r="B35" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="48" t="str">
+      <c r="C35" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Órdenes de compra e integración SGM</v>
       </c>
@@ -16144,7 +16144,7 @@
       <c r="B36" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C36" s="47" t="str">
+      <c r="C36" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Recepción en sucursal y convivencia SGM</v>
       </c>
@@ -16197,7 +16197,7 @@
       <c r="B37" s="16" t="s">
         <v>66</v>
       </c>
-      <c r="C37" s="48" t="str">
+      <c r="C37" s="46" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Inventarios y ajustes</v>
       </c>
@@ -16250,7 +16250,7 @@
       <c r="B38" s="13" t="s">
         <v>78</v>
       </c>
-      <c r="C38" s="47" t="str">
+      <c r="C38" s="45" t="str">
         <f>VLOOKUP(T_UAT[[#This Row],[Módulo]],T_Asignaciones[[ID]:[Capacidad B1]],2,FALSE)</f>
         <v>Stock, conciliación y observabilidad</v>
       </c>
@@ -16298,10 +16298,10 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="S6:S38">
-    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="Fallido"/>
+    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="Fallido"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="V6:V38">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="Falta"/>
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Falta"/>
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation type="list" sqref="S6:S38" xr:uid="{00000000-0002-0000-0500-000000000000}">
@@ -16734,7 +16734,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="H6:H23">
-    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="Fuera"/>
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Fuera"/>
   </conditionalFormatting>
   <dataValidations count="1">
     <dataValidation type="list" sqref="H6:H23" xr:uid="{00000000-0002-0000-0600-000000000000}">
@@ -16782,11 +16782,11 @@
       <c r="L1" s="1"/>
     </row>
     <row r="2" spans="1:12" ht="24.95" customHeight="1">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="47" t="s">
         <v>800</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -16798,12 +16798,12 @@
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" ht="20.100000000000001" customHeight="1">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="48" t="s">
         <v>801</v>
       </c>
-      <c r="B3" s="46"/>
-      <c r="C3" s="46"/>
-      <c r="D3" s="46"/>
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="48"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>

</xml_diff>